<commit_message>
CLP 2025: dados reais do MT a partir do print do site oficial
- Atualiza clp_ranking com 9 indicadores do Pilar Solidez Fiscal:
  Taxa Inv 5º, Regra Ouro 2º, Solvência Fiscal 1º (líder),
  Suc. Planejamento 20º, Dep. Fiscal 7º, Result. Primário 25º,
  Gasto com Pessoal 10º. Índice de Liquidez e Poupança Corrente
  ficam como "ND" (não visíveis no print).
- clp_meta: pos_geral atualizado para "3º (↓1 vs 2024)" e ano_ranking 2025
- index.html: título do card CLP atualizado para "Pilar Solidez Fiscal (2025)"
</commit_message>
<xml_diff>
--- a/manual/panorama_manual.xlsx
+++ b/manual/panorama_manual.xlsx
@@ -10,9 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kpis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="capag" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pessoal" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clp_ranking" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clp_meta" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="investimentos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="investimentos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clp_ranking" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clp_meta" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +476,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>amber</t>
@@ -494,7 +493,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>green</t>
@@ -512,7 +510,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>green</t>
@@ -588,14 +585,11 @@
           <t>Endividamento (% da RCL)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Para nota A: &lt; 60%</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Mede a dívida consolidada do estado em relação à receita corrente líquida. Quanto menor, melhor. Abaixo de 60% da RCL = nota A.</t>
@@ -608,14 +602,11 @@
           <t>Poupança Corrente (Despesa/Receita)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Para nota B: &lt; 95%</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Mede quanto das receitas correntes é consumido pelas despesas correntes. Acima de 95% significa que o estado gasta quase tudo que arrecada só para se manter, sem sobrar para investir.</t>
@@ -628,14 +619,11 @@
           <t>Liquidez Relativa (Dívida/RCL)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Para nota A: ≥ 5%</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Mede se o estado tem recursos disponíveis em caixa para honrar suas obrigações de curto prazo.</t>
@@ -723,104 +711,399 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>indicador</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>posicao</t>
+          <t>pct</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>conceito</t>
+          <t>ranking</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>destaque</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Taxa de Investimentos</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Investimento liquidado dividido pela receita corrente líquida.</t>
-        </is>
+        <v>3.1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sucesso Planejamento Orçamentário</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Despesa liquidada pela despesa total atualizada (dotação orçamentária).</t>
-        </is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Resultado Primário</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Diferença entre receita primária realizada e despesa primária empenhada no ano, dividida pelo PIB nominal do estado.</t>
-        </is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Índice de Liquidez</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Obrigações financeiras divididas pelo caixa bruto. Quanto maior o indicador, pior.</t>
-        </is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Regra de Ouro</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="C12" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="C16" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="C18" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>7</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>14</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="C27" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Diferença entre despesas de capital empenhadas e receita de operações de crédito, dividida pela receita corrente líquida.</t>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>17</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Média BR</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>green</t>
         </is>
       </c>
     </row>
@@ -835,42 +1118,162 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>chave</t>
+          <t>indicador</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>posicao</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>conceito</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pos_geral</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1º (Solvência Fiscal)</t>
+          <t>Taxa de Investimentos</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Investimento liquidado dividido pela receita corrente líquida.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pos_geral_obs</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MT lidera nacionalmente o indicador de Solvência Fiscal do Ranking CLP 2024.</t>
+          <t>Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Diferença entre despesas de capital empenhadas e receita de operações de crédito, dividida pela receita corrente líquida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Solvência Fiscal</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mede a relação entre dívida pública e receita corrente líquida ajustada — quanto menor, melhor. MT lidera o ranking nacional neste indicador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sucesso do Planejamento Orçamentário</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Despesa liquidada dividida pela despesa total atualizada (dotação orçamentária).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dependência Fiscal</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mede o quanto o ente depende de transferências para sustentar suas despesas correntes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Resultado Primário</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>25</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Diferença entre receita primária realizada e despesa primária empenhada no ano, dividida pelo PIB nominal do estado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Gasto com Pessoal</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Despesa total com pessoal sobre a Receita Corrente Líquida (cumprimento da LRF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Índice de Liquidez</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Obrigações financeiras divididas pelo caixa bruto. Quanto maior o indicador, pior. Valor não visível no print de origem — preencher manualmente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Poupança Corrente</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Despesas correntes sobre receitas correntes — quanto maior, menos margem para investir. Valor não visível no print de origem — preencher manualmente.</t>
         </is>
       </c>
     </row>
@@ -885,399 +1288,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>estado</t>
+          <t>chave</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>pct</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ranking</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>destaque</t>
+          <t>valor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27</v>
+          <t>pos_geral</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3º (↓1 vs 2024)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RR</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="C3" t="n">
-        <v>26</v>
+          <t>pos_geral_obs</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MT é 3º no Pilar Solidez Fiscal do Ranking CLP 2025 — caiu uma posição em relação a 2024. Lidera o indicador Solvência Fiscal (1º).</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="C4" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RS</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="C5" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="C7" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="C8" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>DF</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="C9" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>RJ</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="C10" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="C11" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="C12" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>SE</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="C13" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>AP</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="C14" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="C15" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="C16" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="C17" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="C18" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="C19" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="C20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MT</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>7</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>red</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>PB</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="C23" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>GO</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="C24" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="C25" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>14</v>
-      </c>
-      <c r="C26" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>17</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Média BR</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>8.43</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>green</t>
+          <t>ano_ranking</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
     </row>

</xml_diff>